<commit_message>
update code of automating spreadsheets part working with cell styles
</commit_message>
<xml_diff>
--- a/excel_automation/Formulas, Fonts, and Fills.xlsx
+++ b/excel_automation/Formulas, Fonts, and Fills.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,13 +29,32 @@
       <family val="2"/>
       <sz val="11"/>
     </font>
+    <font>
+      <i val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00FF0000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000000FF"/>
+        <bgColor rgb="000000FF"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -50,9 +69,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -470,10 +493,10 @@
           <t>John Smith</t>
         </is>
       </c>
-      <c r="B2" s="1" t="n">
+      <c r="B2" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="5" t="n">
         <v>10</v>
       </c>
       <c r="D2" s="1" t="n">
@@ -493,7 +516,7 @@
           <t>Amit Patel</t>
         </is>
       </c>
-      <c r="B3" s="1" t="n">
+      <c r="B3" s="5" t="n">
         <v>10</v>
       </c>
       <c r="C3" s="1" t="n">
@@ -525,7 +548,7 @@
       <c r="D4" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F4">
@@ -539,13 +562,13 @@
           <t>Sanaa Al Farsi</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="1" t="n">
+      <c r="C5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="1" t="n">
+      <c r="D5" s="5" t="n">
         <v>10</v>
       </c>
       <c r="E5" s="1" t="n">
@@ -589,7 +612,7 @@
       <c r="C7" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="1" t="n">
+      <c r="D7" s="3" t="n">
         <v>4</v>
       </c>
       <c r="E7" s="1" t="n">
@@ -606,16 +629,16 @@
           <t>James Wilson</t>
         </is>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B8" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="C8" s="1" t="n">
+      <c r="C8" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="1" t="n">
+      <c r="D8" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="5" t="n">
         <v>10</v>
       </c>
       <c r="F8">
@@ -629,7 +652,7 @@
           <t>Maria Rodriguez</t>
         </is>
       </c>
-      <c r="B9" s="1" t="n">
+      <c r="B9" s="3" t="n">
         <v>3</v>
       </c>
       <c r="C9" s="1" t="n">
@@ -655,10 +678,10 @@
       <c r="B10" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="1" t="n">
+      <c r="C10" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="1" t="n">
+      <c r="D10" s="5" t="n">
         <v>10</v>
       </c>
       <c r="E10" s="1" t="inlineStr"/>
@@ -676,7 +699,7 @@
       <c r="B11" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="C11" s="1" t="n">
+      <c r="C11" s="3" t="n">
         <v>4</v>
       </c>
       <c r="D11" s="1" t="n">

</xml_diff>